<commit_message>
Update Japanese verb conjugation table
</commit_message>
<xml_diff>
--- a/Studymaterials/日本語用言活用対応表.xlsx
+++ b/Studymaterials/日本語用言活用対応表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nakag\Desktop\GitHub\Myownproject\Studymaterials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D4363B-8C05-4CD9-9D5F-776BAC6E567E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B83648D-969B-47AD-9C6E-0BBABFDB1AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{9E35DED3-8AFA-45C8-BA1E-7705890B6353}"/>
   </bookViews>
@@ -448,62 +448,6 @@
     <phoneticPr fontId="2"/>
   </si>
   <si>
-    <t>「堂々たり」の現代口語訳は「堂々と」という副詞とも考えられる。
-ここでは、用言としての機能をも耐えるために「堂々としている」とした。これは副詞「堂々と」＋サ変動詞「し」の連用形＋助詞「で」＋補助動詞「いる」から構成される。</t>
-    <rPh sb="1" eb="3">
-      <t>ドウドウ</t>
-    </rPh>
-    <rPh sb="7" eb="9">
-      <t>ゲンダイ</t>
-    </rPh>
-    <rPh sb="9" eb="12">
-      <t>コウゴヤク</t>
-    </rPh>
-    <rPh sb="14" eb="16">
-      <t>ドウドウ</t>
-    </rPh>
-    <rPh sb="21" eb="23">
-      <t>フクシ</t>
-    </rPh>
-    <rPh sb="25" eb="26">
-      <t>カンガ</t>
-    </rPh>
-    <rPh sb="37" eb="39">
-      <t>ヨウゲン</t>
-    </rPh>
-    <rPh sb="43" eb="45">
-      <t>キノウ</t>
-    </rPh>
-    <rPh sb="47" eb="48">
-      <t>タ</t>
-    </rPh>
-    <rPh sb="54" eb="56">
-      <t>ドウドウ</t>
-    </rPh>
-    <rPh sb="69" eb="71">
-      <t>フクシ</t>
-    </rPh>
-    <rPh sb="72" eb="74">
-      <t>ドウドウ</t>
-    </rPh>
-    <rPh sb="78" eb="81">
-      <t>ヘンドウシ</t>
-    </rPh>
-    <rPh sb="85" eb="88">
-      <t>レンヨウケイ</t>
-    </rPh>
-    <rPh sb="89" eb="91">
-      <t>ジョシ</t>
-    </rPh>
-    <rPh sb="95" eb="99">
-      <t>ホジョドウシ</t>
-    </rPh>
-    <rPh sb="105" eb="107">
-      <t>コウセイ</t>
-    </rPh>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>口語の
 活用</t>
     <phoneticPr fontId="2"/>
@@ -693,6 +637,62 @@
     </rPh>
     <rPh sb="8" eb="12">
       <t>フクゴウドウシ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>「堂々たり」の現代口語訳は「堂々と」という副詞とも考えられる。
+ここでは、用言としての機能を持たせるために「堂々としている」とした。これは副詞「堂々と」＋サ変動詞「し」の連用形＋助詞「で」＋補助動詞「いる」から構成される。</t>
+    <rPh sb="1" eb="3">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ゲンダイ</t>
+    </rPh>
+    <rPh sb="9" eb="12">
+      <t>コウゴヤク</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="21" eb="23">
+      <t>フクシ</t>
+    </rPh>
+    <rPh sb="25" eb="26">
+      <t>カンガ</t>
+    </rPh>
+    <rPh sb="37" eb="39">
+      <t>ヨウゲン</t>
+    </rPh>
+    <rPh sb="43" eb="45">
+      <t>キノウ</t>
+    </rPh>
+    <rPh sb="46" eb="47">
+      <t>モ</t>
+    </rPh>
+    <rPh sb="54" eb="56">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="69" eb="71">
+      <t>フクシ</t>
+    </rPh>
+    <rPh sb="72" eb="74">
+      <t>ドウドウ</t>
+    </rPh>
+    <rPh sb="78" eb="81">
+      <t>ヘンドウシ</t>
+    </rPh>
+    <rPh sb="85" eb="88">
+      <t>レンヨウケイ</t>
+    </rPh>
+    <rPh sb="89" eb="91">
+      <t>ジョシ</t>
+    </rPh>
+    <rPh sb="95" eb="99">
+      <t>ホジョドウシ</t>
+    </rPh>
+    <rPh sb="105" eb="107">
+      <t>コウセイ</t>
     </rPh>
     <phoneticPr fontId="2"/>
   </si>
@@ -1215,6 +1215,55 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1227,55 +1276,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1593,35 +1593,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="22" customHeight="1">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="18" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="18" t="s">
+      <c r="D1" s="36"/>
+      <c r="E1" s="36"/>
+      <c r="F1" s="36"/>
+      <c r="G1" s="36"/>
+      <c r="H1" s="36"/>
+      <c r="I1" s="36"/>
+      <c r="J1" s="36"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="20"/>
-      <c r="N1" s="18" t="s">
+      <c r="M1" s="37"/>
+      <c r="N1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="O1" s="21"/>
+      <c r="O1" s="38"/>
     </row>
     <row r="2" spans="1:17" ht="58" customHeight="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="23"/>
+      <c r="B2" s="25"/>
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1661,18 +1661,18 @@
       <c r="O2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="P2" s="29" t="s">
+      <c r="P2" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="Q2" s="24" t="s">
-        <v>150</v>
+      <c r="Q2" s="16" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="75" customHeight="1">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="23"/>
+      <c r="B3" s="25"/>
       <c r="C3" s="1" t="s">
         <v>20</v>
       </c>
@@ -1712,14 +1712,14 @@
       <c r="O3" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="P3" s="30"/>
-      <c r="Q3" s="25"/>
+      <c r="P3" s="22"/>
+      <c r="Q3" s="17"/>
     </row>
     <row r="4" spans="1:17" ht="58" customHeight="1">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="23"/>
+      <c r="B4" s="25"/>
       <c r="C4" s="1" t="s">
         <v>34</v>
       </c>
@@ -1759,11 +1759,11 @@
       <c r="O4" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="P4" s="30"/>
-      <c r="Q4" s="25"/>
+      <c r="P4" s="22"/>
+      <c r="Q4" s="17"/>
     </row>
     <row r="5" spans="1:17" ht="44" customHeight="1">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="28" t="s">
         <v>45</v>
       </c>
       <c r="B5" s="14" t="s">
@@ -1808,11 +1808,11 @@
       <c r="O5" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="P5" s="30"/>
-      <c r="Q5" s="25"/>
+      <c r="P5" s="22"/>
+      <c r="Q5" s="17"/>
     </row>
     <row r="6" spans="1:17" ht="44" customHeight="1">
-      <c r="A6" s="35"/>
+      <c r="A6" s="29"/>
       <c r="B6" s="14" t="s">
         <v>58</v>
       </c>
@@ -1855,11 +1855,11 @@
       <c r="O6" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="P6" s="30"/>
-      <c r="Q6" s="25"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="17"/>
     </row>
     <row r="7" spans="1:17" ht="44" customHeight="1">
-      <c r="A7" s="35"/>
+      <c r="A7" s="29"/>
       <c r="B7" s="14" t="s">
         <v>64</v>
       </c>
@@ -1902,11 +1902,11 @@
       <c r="O7" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="P7" s="30"/>
-      <c r="Q7" s="25"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="17"/>
     </row>
     <row r="8" spans="1:17" ht="44" customHeight="1">
-      <c r="A8" s="35"/>
+      <c r="A8" s="29"/>
       <c r="B8" s="14" t="s">
         <v>69</v>
       </c>
@@ -1949,11 +1949,11 @@
       <c r="O8" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="P8" s="30"/>
-      <c r="Q8" s="25"/>
+      <c r="P8" s="22"/>
+      <c r="Q8" s="17"/>
     </row>
     <row r="9" spans="1:17" ht="44" customHeight="1">
-      <c r="A9" s="35"/>
+      <c r="A9" s="29"/>
       <c r="B9" s="14" t="s">
         <v>75</v>
       </c>
@@ -1996,11 +1996,11 @@
       <c r="O9" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="P9" s="30"/>
-      <c r="Q9" s="25"/>
+      <c r="P9" s="22"/>
+      <c r="Q9" s="17"/>
     </row>
     <row r="10" spans="1:17" ht="44" customHeight="1">
-      <c r="A10" s="35"/>
+      <c r="A10" s="29"/>
       <c r="B10" s="15" t="s">
         <v>83</v>
       </c>
@@ -2039,19 +2039,19 @@
       <c r="O10" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="P10" s="30"/>
-      <c r="Q10" s="25"/>
+      <c r="P10" s="22"/>
+      <c r="Q10" s="17"/>
     </row>
     <row r="11" spans="1:17" ht="135" customHeight="1" thickBot="1">
-      <c r="A11" s="37" t="s">
+      <c r="A11" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="B11" s="38"/>
+      <c r="B11" s="32"/>
       <c r="C11" s="7" t="s">
         <v>91</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>92</v>
@@ -2063,7 +2063,7 @@
         <v>94</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>95</v>
@@ -2086,14 +2086,14 @@
       <c r="O11" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="26"/>
+      <c r="P11" s="23"/>
+      <c r="Q11" s="18"/>
     </row>
     <row r="12" spans="1:17" ht="75" customHeight="1">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="B12" s="28"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="9" t="s">
         <v>20</v>
       </c>
@@ -2133,17 +2133,17 @@
       <c r="O12" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="P12" s="29" t="s">
-        <v>111</v>
+      <c r="P12" s="21" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="62" customHeight="1">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="B13" s="25"/>
+      <c r="C13" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B13" s="23"/>
-      <c r="C13" s="1" t="s">
-        <v>113</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>6</v>
@@ -2152,16 +2152,16 @@
         <v>6</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>8</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>12</v>
@@ -2169,23 +2169,23 @@
       <c r="K13" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="L13" s="32" t="s">
+      <c r="L13" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="M13" s="33"/>
+      <c r="M13" s="27"/>
       <c r="N13" s="1" t="s">
         <v>3</v>
       </c>
       <c r="O13" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="P13" s="30"/>
+        <v>113</v>
+      </c>
+      <c r="P13" s="22"/>
     </row>
     <row r="14" spans="1:17" ht="85" customHeight="1">
-      <c r="A14" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="23"/>
+      <c r="A14" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" s="25"/>
       <c r="C14" s="1" t="s">
         <v>34</v>
       </c>
@@ -2193,13 +2193,13 @@
         <v>35</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>37</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>39</v>
@@ -2223,19 +2223,19 @@
         <v>43</v>
       </c>
       <c r="O14" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="P14" s="30"/>
+        <v>117</v>
+      </c>
+      <c r="P14" s="22"/>
     </row>
     <row r="15" spans="1:17" ht="44" customHeight="1">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="28" t="s">
         <v>45</v>
       </c>
       <c r="B15" s="14" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>48</v>
@@ -2244,44 +2244,44 @@
         <v>48</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>48</v>
       </c>
       <c r="H15" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I15" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="J15" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>122</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>54</v>
       </c>
       <c r="L15" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="N15" s="3" t="s">
         <v>123</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>124</v>
       </c>
       <c r="O15" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="P15" s="30"/>
+      <c r="P15" s="22"/>
     </row>
     <row r="16" spans="1:17" ht="44" customHeight="1">
-      <c r="A16" s="35"/>
+      <c r="A16" s="29"/>
       <c r="B16" s="14" t="s">
         <v>58</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>48</v>
@@ -2290,16 +2290,16 @@
         <v>48</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>48</v>
       </c>
       <c r="H16" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="I16" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>127</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>61</v>
@@ -2308,21 +2308,21 @@
         <v>49</v>
       </c>
       <c r="L16" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="M16" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>129</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>130</v>
       </c>
       <c r="O16" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="P16" s="30"/>
+      <c r="P16" s="22"/>
     </row>
     <row r="17" spans="1:16" ht="44" customHeight="1">
-      <c r="A17" s="35"/>
+      <c r="A17" s="29"/>
       <c r="B17" s="14" t="s">
         <v>64</v>
       </c>
@@ -2354,21 +2354,21 @@
         <v>70</v>
       </c>
       <c r="L17" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="N17" s="3" t="s">
         <v>131</v>
-      </c>
-      <c r="M17" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>132</v>
       </c>
       <c r="O17" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="P17" s="30"/>
+      <c r="P17" s="22"/>
     </row>
     <row r="18" spans="1:16" ht="44" customHeight="1">
-      <c r="A18" s="35"/>
+      <c r="A18" s="29"/>
       <c r="B18" s="14" t="s">
         <v>69</v>
       </c>
@@ -2400,10 +2400,10 @@
         <v>70</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M18" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="N18" s="3" t="s">
         <v>52</v>
@@ -2411,12 +2411,12 @@
       <c r="O18" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="P18" s="30"/>
+      <c r="P18" s="22"/>
     </row>
     <row r="19" spans="1:16" ht="44" customHeight="1">
-      <c r="A19" s="35"/>
+      <c r="A19" s="29"/>
       <c r="B19" s="14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>50</v>
@@ -2457,10 +2457,10 @@
       <c r="O19" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="P19" s="30"/>
+      <c r="P19" s="22"/>
     </row>
     <row r="20" spans="1:16" ht="44" customHeight="1">
-      <c r="A20" s="36"/>
+      <c r="A20" s="30"/>
       <c r="B20" s="14" t="s">
         <v>83</v>
       </c>
@@ -2468,16 +2468,16 @@
         <v>50</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="F20" s="3" t="s">
         <v>76</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>76</v>
@@ -2486,67 +2486,72 @@
         <v>87</v>
       </c>
       <c r="J20" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="K20" s="3" t="s">
         <v>135</v>
-      </c>
-      <c r="K20" s="3" t="s">
-        <v>136</v>
       </c>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
       <c r="N20" s="3"/>
       <c r="O20" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="P20" s="30"/>
+        <v>136</v>
+      </c>
+      <c r="P20" s="22"/>
     </row>
     <row r="21" spans="1:16" ht="135" customHeight="1" thickBot="1">
-      <c r="A21" s="37" t="s">
+      <c r="A21" s="31" t="s">
+        <v>137</v>
+      </c>
+      <c r="B21" s="32"/>
+      <c r="C21" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="B21" s="38"/>
-      <c r="C21" s="7" t="s">
+      <c r="D21" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="E21" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="F21" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="F21" s="7" t="s">
+      <c r="G21" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="G21" s="7" t="s">
+      <c r="H21" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="H21" s="7" t="s">
+      <c r="I21" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="J21" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="J21" s="7" t="s">
+      <c r="K21" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="K21" s="7" t="s">
+      <c r="L21" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="L21" s="7" t="s">
+      <c r="M21" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="N21" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="M21" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="N21" s="7" t="s">
+      <c r="O21" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="O21" s="8" t="s">
-        <v>149</v>
-      </c>
-      <c r="P21" s="31"/>
+      <c r="P21" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:K1"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="N1:O1"/>
+    <mergeCell ref="A2:B2"/>
     <mergeCell ref="Q2:Q11"/>
     <mergeCell ref="A12:B12"/>
     <mergeCell ref="P12:P21"/>
@@ -2560,11 +2565,6 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:A10"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C1:K1"/>
-    <mergeCell ref="L1:M1"/>
-    <mergeCell ref="N1:O1"/>
-    <mergeCell ref="A2:B2"/>
   </mergeCells>
   <phoneticPr fontId="2"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>